<commit_message>
feat(vehicles): add sub_department + populate xlsx with real fleet data
* Migration adds vehicles.sub_department (text, nullable).
* Vehicle TS interface gains sub_department.
* VehicleHistoryPage shows it next to department in the header.
* Excel generator now emits a 4-column vehicles.xlsx (added "תת מחלקה")
  pre-populated with 25 vehicles supplied by the user (2026-05-03):
    • סיור (6)
    • מנהלה (6)
    • אושקוש סולר (2)
    • FMTV (4)
    • אושקוש מרום, אמבולנס, האמר כתקל / בקש / רקש,
      FMTV חלפים, ריאו מים (1 each)
  All entries: profession=רכב, department=רכב.

The labels following the vehicle numbers in the user's source list
(e.g. "סיור 1", "חרמש", "נחשונים") are NOT captured — no column
exists for them yet. Will add if requested.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/worker_templates/vehicles.xlsx
+++ b/worker_templates/vehicles.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,10 +29,6 @@
     <font>
       <b val="1"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00888888"/>
     </font>
     <font>
       <b val="1"/>
@@ -65,13 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -440,12 +435,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -464,85 +460,559 @@
           <t>מחלקה</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>תת מחלקה</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>12-345-67</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>רכב</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>מחלקת תחזוקה</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>705-164</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>סיור</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>23-456-78</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>חשמל</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>מחלקת חשמל</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>705-135</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>סיור</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>34-567-89</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>רכב</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>705-430</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>סיור</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>45-678-90</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>אופטיקה</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>מחלקת אופטיקה</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>705-476</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>סיור</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>56-789-01</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>חשמל</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>מחלקת חשמל</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>705-194</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>סיור</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>705-416</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>סיור</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>706-677</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>מנהלה</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>706-682</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>מנהלה</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>706-713</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>מנהלה</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>706-714</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>מנהלה</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>706-615</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>מנהלה</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>706-600</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>מנהלה</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>707-156</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>אושקוש סולר</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>707-267</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>אושקוש סולר</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>990-084</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>FMTV</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>990-088</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>FMTV</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>990-082</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>FMTV</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>990-405</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>FMTV</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>684-663</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>אושקוש מרום</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>561-414</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>אמבולנס</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>705-285</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>האמר כתקל</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>700-402</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>האמר בקש</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>706-549</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>האמר רקש</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>990-919</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>FMTV חלפים</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>676-741</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ריאו מים</t>
         </is>
       </c>
     </row>
@@ -557,69 +1027,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>הוראות מילוי</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>טבלה זו רושמת את הרכבים והציוד שמטופלים במערכת.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>כל רכב בשורה נפרדת.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr"/>
+      <c r="A5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>עמודות:</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • מספר רכב — מספר/מזהה ייחודי. דוגמה: "12-345-67" (מספר רישוי) או "G500-001" (מזהה פנימי).</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • מספר רכב — מספר/מזהה ייחודי. דוגמה: "705-164" או "G500-001".</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • מקצוע — שם המקצוע שאחראי על הרכב. חייב להתאים לאחד הערכים שיופיעו בעמודת "מקצוע" ב-employees.xlsx.</t>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • מקצוע — שם המקצוע שאחראי על הרכב. חייב להתאים לאחד הערכים שיופיעו בעמודת "מקצוע" ב-employees.xlsx (למשל: "רכב", "חשמל", "אופטיקה").</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  • מחלקה — מחלקה ארגונית שאליה שייך הרכב. אופציונלי.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr"/>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • תת מחלקה — קטגוריה משנית בתוך המחלקה (למשל "סיור", "מנהלה", "FMTV", "אמבולנס"). אופציונלי.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>הערה: סוג הרכב הוא הקובע איזה צוות טכנאים רואה את הקריאות לרכב הזה.</t>
         </is>

</xml_diff>

<commit_message>
data(vehicles): apply user labels to sub_department + strip dashes
* New scripts/update_vehicles.py: idempotent in-place update of
  worker_templates/vehicles.xlsx. Uses LABEL_MAP for the 25 רכב
  vehicles (e.g. 705430 -> 'נחשונים'); leaves any other rows the
  user added intact except for normalizing dashes out of the
  vehicle_number column.

* vehicles.xlsx after run:
    - 25 מספרים נוקו (705-164 -> 705164, etc.)
    - 12 שורות עודכנו עם תוויות (סיור 1/2, נחשונים, חרמש,
      מג״ד, רפואה, פלוגה מ/ל/כ, חרמש 1)
    - 13 שורות בלי תוויות שמרו על הקטגוריה כסאב (FMTV, אושקוש
      סולר/מרום, אמבולנס, האמרים, FMTV חלפים, ריאו מים)
    - 15 שורות טנק שהמשתמש הוסיף הושארו כמות שהן

Going forward vehicles.xlsx is the source of truth — generate_excel_
templates.py is no longer the canonical writer for this file.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/worker_templates/vehicles.xlsx
+++ b/worker_templates/vehicles.xlsx
@@ -2,23 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הוראות" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,12 +26,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <sz val="12"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <i val="1"/>
+      <color rgb="FF888888"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -44,8 +54,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
-        <bgColor rgb="00DBEAFE"/>
+        <fgColor rgb="FFDBEAFE"/>
+        <bgColor rgb="FFDBEAFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -70,9 +80,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -435,12 +446,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D41"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="2" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -469,7 +479,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>705-164</t>
+          <t>705164</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -484,14 +494,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>סיור</t>
+          <t>סיור 1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>705-135</t>
+          <t>705135</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -506,14 +516,14 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>סיור</t>
+          <t>סיור 2</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>705-430</t>
+          <t>705430</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -528,14 +538,14 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>סיור</t>
+          <t>נחשונים</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>705-476</t>
+          <t>705476</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -550,14 +560,14 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>סיור</t>
+          <t>חרמש</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>705-194</t>
+          <t>705194</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -572,14 +582,14 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>סיור</t>
+          <t>מג״ד</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>705-416</t>
+          <t>705416</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -594,14 +604,14 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>סיור</t>
+          <t>חרמש</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>706-677</t>
+          <t>706677</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -616,14 +626,14 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>מנהלה</t>
+          <t>רפואה</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>706-682</t>
+          <t>706682</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -638,14 +648,14 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>מנהלה</t>
+          <t>פלוגה מ</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>706-713</t>
+          <t>706713</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -660,14 +670,14 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>מנהלה</t>
+          <t>חרמש 1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>706-714</t>
+          <t>706714</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -682,14 +692,14 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>מנהלה</t>
+          <t>נחשונים</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>706-615</t>
+          <t>706615</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -704,14 +714,14 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>מנהלה</t>
+          <t>פלוגה ל</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>706-600</t>
+          <t>706600</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -726,14 +736,14 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>מנהלה</t>
+          <t>פלוגה כ</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>707-156</t>
+          <t>707156</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -755,7 +765,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>707-267</t>
+          <t>707267</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -777,7 +787,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>990-084</t>
+          <t>990084</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -799,7 +809,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>990-088</t>
+          <t>990088</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -821,7 +831,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>990-082</t>
+          <t>990082</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -843,7 +853,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>990-405</t>
+          <t>990405</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -865,7 +875,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>684-663</t>
+          <t>684663</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -887,7 +897,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>561-414</t>
+          <t>561414</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -909,7 +919,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>705-285</t>
+          <t>705285</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -931,7 +941,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>700-402</t>
+          <t>700402</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -953,7 +963,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>706-549</t>
+          <t>706549</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -975,7 +985,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>990-919</t>
+          <t>990919</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -997,7 +1007,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>676-741</t>
+          <t>676741</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1013,6 +1023,306 @@
       <c r="D26" t="inlineStr">
         <is>
           <t>ריאו מים</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>835063</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>טנק</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>ל</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>ל</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>835423</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>טנק</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>ל</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>ל</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>835033</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>טנק</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>ל</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>ל</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>835150</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>טנק</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>ל</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>ל</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>835083</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>טנק</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>כ</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>כ</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>835361</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>טנק</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>כ</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>כ</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>835304</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>טנק</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>כ</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>כ</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>835152</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>טנק</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>כ</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>כ</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>835317</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>טנק</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>כ</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>כ</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>835165</v>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>טנק</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>כ</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>כ</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>835109</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>טנק</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>מ</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>מ</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n">
+        <v>835145</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>טנק</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>מ</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>מ</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>835146</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>טנק</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>מ</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>מ</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n">
+        <v>835372</v>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>טנק</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>מ</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>מ</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>835399</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>טנק</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>מ</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>מ</t>
         </is>
       </c>
     </row>
@@ -1028,26 +1338,26 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="19" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
           <t>הוראות מילוי</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>טבלה זו רושמת את הרכבים והציוד שמטופלים במערכת.</t>
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>כל רכב בשורה נפרדת.</t>
@@ -1055,37 +1365,37 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
+      <c r="A5" s="3" t="n"/>
+    </row>
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>עמודות:</t>
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  • מספר רכב — מספר/מזהה ייחודי. דוגמה: "705-164" או "G500-001".</t>
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  • מקצוע — שם המקצוע שאחראי על הרכב. חייב להתאים לאחד הערכים שיופיעו בעמודת "מקצוע" ב-employees.xlsx (למשל: "רכב", "חשמל", "אופטיקה").</t>
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  • מחלקה — מחלקה ארגונית שאליה שייך הרכב. אופציונלי.</t>
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  • תת מחלקה — קטגוריה משנית בתוך המחלקה (למשל "סיור", "מנהלה", "FMTV", "אמבולנס"). אופציונלי.</t>
@@ -1093,9 +1403,9 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
+      <c r="A11" s="3" t="n"/>
+    </row>
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>הערה: סוג הרכב הוא הקובע איזה צוות טכנאים רואה את הקריאות לרכב הזה.</t>

</xml_diff>